<commit_message>
Apply Rozum branding and remove popup notes from lecturer workbooks
</commit_message>
<xml_diff>
--- a/Тематика для рассылки/Пробная версия/01_Анкета_лектора_ПРОБНАЯ.xlsx
+++ b/Тематика для рассылки/Пробная версия/01_Анкета_лектора_ПРОБНАЯ.xlsx
@@ -42,30 +42,30 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00221F1F"/>
       <sz val="20"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="0017324D"/>
+      <color rgb="00221F1F"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="0017324D"/>
+      <color rgb="00221F1F"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00087F8C"/>
+      <color rgb="00008685"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00087F8C"/>
+      <color rgb="00008685"/>
       <sz val="11"/>
       <u val="single"/>
     </font>
@@ -83,11 +83,11 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="0017324D"/>
+      <color rgb="00221F1F"/>
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -96,37 +96,42 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0017324D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EAF3F6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF3C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF0DA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F7FA"/>
+        <fgColor rgb="00F0F8F4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00087F8C"/>
+        <fgColor rgb="00E5F5EF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F5F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00221F1F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0026BBA8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0040B870"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00008685"/>
       </patternFill>
     </fill>
   </fills>
@@ -140,14 +145,14 @@
     </border>
     <border>
       <bottom style="thin">
-        <color rgb="00D0AD48"/>
+        <color rgb="0040B870"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
@@ -178,56 +183,108 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <color rgb="00221F1F"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00221F1F"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="medium">
+          <color rgb="0026BBA8"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00E2F2E9"/>
+          <fgColor rgb="00FFFFFF"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFD9B3"/>
+          <fgColor rgb="00F0F8F4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00DDF2E5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C9EBDF"/>
         </patternFill>
       </fill>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="RozumTable" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="RozumTable" pivot="0" table="1">
+      <tableStyleElement type="wholeTable" dxfId="0"/>
+      <tableStyleElement type="headerRow" dxfId="1"/>
+      <tableStyleElement type="firstRowStripe" size="1" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" size="1" dxfId="3"/>
+    </tableStyle>
+  </tableStyles>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -299,96 +356,94 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Инструкция</author>
-    <author>Содержание из программы</author>
-  </authors>
-  <commentList>
-    <comment ref="F4" authorId="0" shapeId="0">
-      <text>
-        <t>Введите дату заполнения, например 15.10.2026. При желании её можно оставить пустой.</t>
-      </text>
-    </comment>
-    <comment ref="B11" authorId="1" shapeId="0">
-      <text>
-        <t>Киберпреступность. Международный опыт противодействия киберпреступности. Построение системы обеспечения кибербезопасности в Республике Беларусь и Российской Федерации.
-Источник: РАЗДЕЛ I Методология расследования инцидентов., Тема 1. Кибербезопасность, информационная безопасность, защита информации. Опыт противодействия киберпреступности (на примере Республики Беларусь и Российской Федерации) (1 час лекции).</t>
-      </text>
-    </comment>
-    <comment ref="B12" authorId="1" shapeId="0">
-      <text>
-        <t>Типовая корпоративная информационная система (далее – ИС), которая представляет собой комплекс программных и аппаратных средств, предназначенных для автоматизации бизнес-процессов в организации. Основные компоненты системы, структура, принципы построения и внедрения.
-Источник: РАЗДЕЛ I Методология расследования инцидентов., Тема 2. Типовая корпоративная информационная система (1 час лекции).</t>
-      </text>
-    </comment>
-    <comment ref="B13" authorId="1" shapeId="0">
-      <text>
-        <t>Матрица MITRE ATT&amp;CK. Модель Cyber Kill Chain. Детектирование инцидентов. Работа с индикаторами компрометации.
-Источник: РАЗДЕЛ I Методология расследования инцидентов., Тема 3. Продвинутые кибератаки. Матрица MITRE ATT&amp;CK. Модель Cyber Kill Chain. Индикаторы компрометации (2 часа лекции).</t>
-      </text>
-    </comment>
-    <comment ref="B14" authorId="1" shapeId="0">
-      <text>
-        <t>Эволюция SOC, триада (люди, процессы, технологии), уровни процессов, метрики, роли сотрудников (L1–L3, инженеры, архитектор, руководитель), RACI-матрица, технологии (SIEM, EDR/XDR, SOAR, TI), AI и Agentic SOC.
-Источник: РАЗДЕЛ I Методология расследования инцидентов., Тема 4. Современный SOC (1 час лекции).</t>
-      </text>
-    </comment>
-    <comment ref="B15" authorId="1" shapeId="0">
-      <text>
-        <t>Определения, связанные с информационной безопасностью (ИБ). Этапы жизненного цикла.
-Источник: РАЗДЕЛ I Методология расследования инцидентов., Тема 5. Жизненный цикл информационной безопасности (1 час лекции).</t>
-      </text>
-    </comment>
-    <comment ref="B16" authorId="1" shapeId="0">
-      <text>
-        <t>Инструменты анализа журналов Windows: Event Viewer (фильтры, XML), EvtxECmd (парсинг), Timeline Explorer (просмотр CSV), Get-WinEvent и Wevtutil (консоль), Hayabusa (поиск угроз по Sigma-правилам).
-Источник: РАЗДЕЛ I Методология расследования инцидентов., Тема 7. Анализ журналов и популярных событий Windows (1 час практические занятия).</t>
-      </text>
-    </comment>
-    <comment ref="B17" authorId="1" shapeId="0">
-      <text>
-        <t>Типовая корпоративная ИС. Основные компоненты ИС, структура, принципы построения и внедрения.
-Концепция доменов в Active Directory (далее – AD). Основные принципы работы доменов, структура, роли контроллера домена.
-Источник: РАЗДЕЛ II «Active Directory» в различных операционных системах., Тема 1. Домены Active Directory. Доменная групповая политика (1 час лекции).</t>
-      </text>
-    </comment>
-    <comment ref="B18" authorId="1" shapeId="0">
-      <text>
-        <t>Процесс аутентификации пользователей и компьютеров в домене Active Directory. Методы аутентификации, протоколы, используемые для передачи учетных данных, механизмы защиты от несанкционированного доступа.
-Источник: РАЗДЕЛ II «Active Directory» в различных операционных системах., Тема 2. Доменная аутентификация. Типовые атаки на протоколы аутентификации (2 часа лекции).</t>
-      </text>
-    </comment>
-    <comment ref="B19" authorId="1" shapeId="0">
-      <text>
-        <t>LDAP (Lightweight Directory Access Protocol): основные понятия и принципы работы LDAP.
-Источник: РАЗДЕЛ II «Active Directory» в различных операционных системах., Тема 4. Введение в LDAP (1 час лекции).</t>
-      </text>
-    </comment>
-    <comment ref="B20" authorId="1" shapeId="0">
-      <text>
-        <t>Создание, изменение, удаление пользователей. Ключевые объектные классы пользователей. Настройка атрибутов пользователей и групп. Использование LDIF для управления. Особенности кодирования в LDIF. Безопасность пользователей.
-Источник: РАЗДЕЛ II «Active Directory» в различных операционных системах., Тема 6. Управление пользователями (1 час лекции).</t>
-      </text>
-    </comment>
-    <comment ref="B21" authorId="1" shapeId="0">
-      <text>
-        <t>Сбор и анализ артефактов инцидента на узлах и в сетевой инфраструктуре. Выявление вектора компрометации и определение последовательности действий нарушителя. Локализация инцидента, сдерживание распространения атаки и восстановление работоспособности сервисов. Отработка типового сценария расследования и реагирования на атаку.
-Источник: РАЗДЕЛ II «Active Directory» в различных операционных системах., Тема 11. Расследование и реагирование на атаку в инфраструктуре (4 часа практические занятия).</t>
-      </text>
-    </comment>
-    <comment ref="B22" authorId="1" shapeId="0">
-      <text>
-        <t>Расследования инцидента «атака вируса-шифровальщика» в инфраструктуре. Идентификация всех этапов атаки, определение всех индикаторов компрометации.
-Сценарий самостоятельной работы:
-анализ результатов выполнения сценария атаки вируса-шифровальщика на киберполигоне;
-закрепление навыков оформления отчетных материалов по результатам расследования инцидента.
-Источник: РАЗДЕЛ III Киберучения., Тема 1. Отработка сценария «атака вируса-шифровальщика» на киберполигоне. Анализ результатов, обсуждение и разбор сценария (4 часа практические занятия, 2 часа самостоятельная работа) [2, 7].</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>57150</colOff>
+      <row>0</row>
+      <rowOff>142875</rowOff>
+    </from>
+    <ext cx="1619250" cy="333375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>57150</colOff>
+      <row>0</row>
+      <rowOff>142875</rowOff>
+    </from>
+    <ext cx="1619250" cy="333375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>57150</colOff>
+      <row>0</row>
+      <rowOff>142875</rowOff>
+    </from>
+    <ext cx="1619250" cy="333375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -402,297 +457,297 @@
     <tableColumn id="5" name="Могу читать"/>
     <tableColumn id="6" name="Комментарий преподавателя"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <tableStyleInfo name="RozumTable" showRowStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
+<ns0:theme xmlns:ns0="http://schemas.openxmlformats.org/drawingml/2006/main" name="Rozum">
+  <ns0:themeElements>
+    <ns0:clrScheme name="Rozum">
+      <ns0:dk1>
+        <ns0:srgbClr val="221F1F"/>
+      </ns0:dk1>
+      <ns0:lt1>
+        <ns0:srgbClr val="FFFFFF"/>
+      </ns0:lt1>
+      <ns0:dk2>
+        <ns0:srgbClr val="221F1F"/>
+      </ns0:dk2>
+      <ns0:lt2>
+        <ns0:srgbClr val="F0F8F4"/>
+      </ns0:lt2>
+      <ns0:accent1>
+        <ns0:srgbClr val="26BBA8"/>
+      </ns0:accent1>
+      <ns0:accent2>
+        <ns0:srgbClr val="40B870"/>
+      </ns0:accent2>
+      <ns0:accent3>
+        <ns0:srgbClr val="008685"/>
+      </ns0:accent3>
+      <ns0:accent4>
+        <ns0:srgbClr val="009763"/>
+      </ns0:accent4>
+      <ns0:accent5>
+        <ns0:srgbClr val="60756C"/>
+      </ns0:accent5>
+      <ns0:accent6>
+        <ns0:srgbClr val="DDF2E5"/>
+      </ns0:accent6>
+      <ns0:hlink>
+        <ns0:srgbClr val="008685"/>
+      </ns0:hlink>
+      <ns0:folHlink>
+        <ns0:srgbClr val="009763"/>
+      </ns0:folHlink>
+    </ns0:clrScheme>
+    <ns0:fontScheme name="Office">
+      <ns0:majorFont>
+        <ns0:latin typeface="Cambria"/>
+        <ns0:ea typeface=""/>
+        <ns0:cs typeface=""/>
+        <ns0:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <ns0:font script="Hang" typeface="맑은 고딕"/>
+        <ns0:font script="Hans" typeface="宋体"/>
+        <ns0:font script="Hant" typeface="新細明體"/>
+        <ns0:font script="Arab" typeface="Times New Roman"/>
+        <ns0:font script="Hebr" typeface="Times New Roman"/>
+        <ns0:font script="Thai" typeface="Tahoma"/>
+        <ns0:font script="Ethi" typeface="Nyala"/>
+        <ns0:font script="Beng" typeface="Vrinda"/>
+        <ns0:font script="Gujr" typeface="Shruti"/>
+        <ns0:font script="Khmr" typeface="MoolBoran"/>
+        <ns0:font script="Knda" typeface="Tunga"/>
+        <ns0:font script="Guru" typeface="Raavi"/>
+        <ns0:font script="Cans" typeface="Euphemia"/>
+        <ns0:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <ns0:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <ns0:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <ns0:font script="Thaa" typeface="MV Boli"/>
+        <ns0:font script="Deva" typeface="Mangal"/>
+        <ns0:font script="Telu" typeface="Gautami"/>
+        <ns0:font script="Taml" typeface="Latha"/>
+        <ns0:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <ns0:font script="Orya" typeface="Kalinga"/>
+        <ns0:font script="Mlym" typeface="Kartika"/>
+        <ns0:font script="Laoo" typeface="DokChampa"/>
+        <ns0:font script="Sinh" typeface="Iskoola Pota"/>
+        <ns0:font script="Mong" typeface="Mongolian Baiti"/>
+        <ns0:font script="Viet" typeface="Times New Roman"/>
+        <ns0:font script="Uigh" typeface="Microsoft Uighur"/>
+      </ns0:majorFont>
+      <ns0:minorFont>
+        <ns0:latin typeface="Calibri"/>
+        <ns0:ea typeface=""/>
+        <ns0:cs typeface=""/>
+        <ns0:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <ns0:font script="Hang" typeface="맑은 고딕"/>
+        <ns0:font script="Hans" typeface="宋体"/>
+        <ns0:font script="Hant" typeface="新細明體"/>
+        <ns0:font script="Arab" typeface="Arial"/>
+        <ns0:font script="Hebr" typeface="Arial"/>
+        <ns0:font script="Thai" typeface="Tahoma"/>
+        <ns0:font script="Ethi" typeface="Nyala"/>
+        <ns0:font script="Beng" typeface="Vrinda"/>
+        <ns0:font script="Gujr" typeface="Shruti"/>
+        <ns0:font script="Khmr" typeface="DaunPenh"/>
+        <ns0:font script="Knda" typeface="Tunga"/>
+        <ns0:font script="Guru" typeface="Raavi"/>
+        <ns0:font script="Cans" typeface="Euphemia"/>
+        <ns0:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <ns0:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <ns0:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <ns0:font script="Thaa" typeface="MV Boli"/>
+        <ns0:font script="Deva" typeface="Mangal"/>
+        <ns0:font script="Telu" typeface="Gautami"/>
+        <ns0:font script="Taml" typeface="Latha"/>
+        <ns0:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <ns0:font script="Orya" typeface="Kalinga"/>
+        <ns0:font script="Mlym" typeface="Kartika"/>
+        <ns0:font script="Laoo" typeface="DokChampa"/>
+        <ns0:font script="Sinh" typeface="Iskoola Pota"/>
+        <ns0:font script="Mong" typeface="Mongolian Baiti"/>
+        <ns0:font script="Viet" typeface="Arial"/>
+        <ns0:font script="Uigh" typeface="Microsoft Uighur"/>
+      </ns0:minorFont>
+    </ns0:fontScheme>
+    <ns0:fmtScheme name="Office">
+      <ns0:fillStyleLst>
+        <ns0:solidFill>
+          <ns0:schemeClr val="phClr"/>
+        </ns0:solidFill>
+        <ns0:gradFill rotWithShape="1">
+          <ns0:gsLst>
+            <ns0:gs pos="0">
+              <ns0:schemeClr val="phClr">
+                <ns0:tint val="50000"/>
+                <ns0:satMod val="300000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="35000">
+              <ns0:schemeClr val="phClr">
+                <ns0:tint val="37000"/>
+                <ns0:satMod val="300000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="100000">
+              <ns0:schemeClr val="phClr">
+                <ns0:tint val="15000"/>
+                <ns0:satMod val="350000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+          </ns0:gsLst>
+          <ns0:lin ang="16200000" scaled="1"/>
+        </ns0:gradFill>
+        <ns0:gradFill rotWithShape="1">
+          <ns0:gsLst>
+            <ns0:gs pos="0">
+              <ns0:schemeClr val="phClr">
+                <ns0:shade val="51000"/>
+                <ns0:satMod val="130000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="80000">
+              <ns0:schemeClr val="phClr">
+                <ns0:shade val="93000"/>
+                <ns0:satMod val="130000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="100000">
+              <ns0:schemeClr val="phClr">
+                <ns0:shade val="94000"/>
+                <ns0:satMod val="135000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+          </ns0:gsLst>
+          <ns0:lin ang="16200000" scaled="0"/>
+        </ns0:gradFill>
+      </ns0:fillStyleLst>
+      <ns0:lnStyleLst>
+        <ns0:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <ns0:solidFill>
+            <ns0:schemeClr val="phClr">
+              <ns0:shade val="95000"/>
+              <ns0:satMod val="105000"/>
+            </ns0:schemeClr>
+          </ns0:solidFill>
+          <ns0:prstDash val="solid"/>
+        </ns0:ln>
+        <ns0:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <ns0:solidFill>
+            <ns0:schemeClr val="phClr"/>
+          </ns0:solidFill>
+          <ns0:prstDash val="solid"/>
+        </ns0:ln>
+        <ns0:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <ns0:solidFill>
+            <ns0:schemeClr val="phClr"/>
+          </ns0:solidFill>
+          <ns0:prstDash val="solid"/>
+        </ns0:ln>
+      </ns0:lnStyleLst>
+      <ns0:effectStyleLst>
+        <ns0:effectStyle>
+          <ns0:effectLst>
+            <ns0:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <ns0:srgbClr val="000000">
+                <ns0:alpha val="38000"/>
+              </ns0:srgbClr>
+            </ns0:outerShdw>
+          </ns0:effectLst>
+        </ns0:effectStyle>
+        <ns0:effectStyle>
+          <ns0:effectLst>
+            <ns0:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <ns0:srgbClr val="000000">
+                <ns0:alpha val="35000"/>
+              </ns0:srgbClr>
+            </ns0:outerShdw>
+          </ns0:effectLst>
+        </ns0:effectStyle>
+        <ns0:effectStyle>
+          <ns0:effectLst>
+            <ns0:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <ns0:srgbClr val="000000">
+                <ns0:alpha val="35000"/>
+              </ns0:srgbClr>
+            </ns0:outerShdw>
+          </ns0:effectLst>
+          <ns0:scene3d>
+            <ns0:camera prst="orthographicFront">
+              <ns0:rot lat="0" lon="0" rev="0"/>
+            </ns0:camera>
+            <ns0:lightRig rig="threePt" dir="t">
+              <ns0:rot lat="0" lon="0" rev="1200000"/>
+            </ns0:lightRig>
+          </ns0:scene3d>
+          <ns0:sp3d>
+            <ns0:bevelT w="63500" h="25400"/>
+          </ns0:sp3d>
+        </ns0:effectStyle>
+      </ns0:effectStyleLst>
+      <ns0:bgFillStyleLst>
+        <ns0:solidFill>
+          <ns0:schemeClr val="phClr"/>
+        </ns0:solidFill>
+        <ns0:gradFill rotWithShape="1">
+          <ns0:gsLst>
+            <ns0:gs pos="0">
+              <ns0:schemeClr val="phClr">
+                <ns0:tint val="40000"/>
+                <ns0:satMod val="350000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="40000">
+              <ns0:schemeClr val="phClr">
+                <ns0:tint val="45000"/>
+                <ns0:shade val="99000"/>
+                <ns0:satMod val="350000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="100000">
+              <ns0:schemeClr val="phClr">
+                <ns0:shade val="20000"/>
+                <ns0:satMod val="255000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+          </ns0:gsLst>
+          <ns0:path path="circle">
+            <ns0:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </ns0:path>
+        </ns0:gradFill>
+        <ns0:gradFill rotWithShape="1">
+          <ns0:gsLst>
+            <ns0:gs pos="0">
+              <ns0:schemeClr val="phClr">
+                <ns0:tint val="80000"/>
+                <ns0:satMod val="300000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="100000">
+              <ns0:schemeClr val="phClr">
+                <ns0:shade val="30000"/>
+                <ns0:satMod val="200000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+          </ns0:gsLst>
+          <ns0:path path="circle">
+            <ns0:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </ns0:path>
+        </ns0:gradFill>
+      </ns0:bgFillStyleLst>
+    </ns0:fmtScheme>
+  </ns0:themeElements>
+  <ns0:objectDefaults/>
+  <ns0:extraClrSchemeLst/>
+</ns0:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00087F8C"/>
+    <tabColor rgb="00008685"/>
     <outlinePr summaryBelow="1" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -707,7 +762,7 @@
     <col width="42" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="44" customHeight="1">
+    <row r="1" ht="52" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>КАКИЕ ТЕМЫ ВЫ ГОТОВЫ ЧИТАТЬ?</t>
@@ -717,7 +772,6 @@
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -782,7 +836,7 @@
     <row r="6" ht="29" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Жёлтые ячейки — для ваших ответов. Пустая отметка означает «не указано». При ответе «Частично» поясните ограничения.</t>
+          <t>Светло-зелёные ячейки — для ваших ответов. Пустая отметка означает «не указано». При ответе «Частично» поясните ограничения.</t>
         </is>
       </c>
       <c r="B6" s="9" t="n"/>
@@ -824,55 +878,63 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="6" customHeight="1">
+      <c r="A9" s="14" t="n"/>
+      <c r="B9" s="14" t="n"/>
+      <c r="C9" s="14" t="n"/>
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="15" t="n"/>
+      <c r="F9" s="15" t="n"/>
+    </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Код темы</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>Тема</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>Программы</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>Содержание</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>Могу читать</t>
         </is>
       </c>
-      <c r="F10" s="14" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>Комментарий преподавателя</t>
         </is>
       </c>
     </row>
     <row r="11" ht="67" customHeight="1">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>T-C7476F67</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Кибербезопасность, информационная безопасность, защита информации. Опыт противодействия киберпреступности (на примере Республики Беларусь и Российской Федерации)</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>ПТИБ (advance)</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>Открыть →</t>
         </is>
@@ -881,22 +943,22 @@
       <c r="F11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>T-AB58E916</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>Типовая корпоративная информационная система</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="19" t="inlineStr">
         <is>
           <t>ПТИБ (advance)</t>
         </is>
       </c>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>Открыть →</t>
         </is>
@@ -905,22 +967,22 @@
       <c r="F12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>T-6F75FEB6</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>Продвинутые кибератаки. Матрица MITRE ATT&amp;CK. Модель Cyber Kill Chain. Индикаторы компрометации</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>ПТИБ (advance)</t>
         </is>
       </c>
-      <c r="D13" s="16" t="inlineStr">
+      <c r="D13" s="18" t="inlineStr">
         <is>
           <t>Открыть →</t>
         </is>
@@ -929,22 +991,22 @@
       <c r="F13" s="6" t="inlineStr"/>
     </row>
     <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>T-05085C3F</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>Современный SOC</t>
         </is>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C14" s="19" t="inlineStr">
         <is>
           <t>ПТИБ (advance)</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D14" s="20" t="inlineStr">
         <is>
           <t>Открыть →</t>
         </is>
@@ -953,22 +1015,22 @@
       <c r="F14" s="6" t="inlineStr"/>
     </row>
     <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>T-8A73AE5B</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Жизненный цикл информационной безопасности</t>
         </is>
       </c>
-      <c r="C15" s="15" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>ПТИБ (advance)</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D15" s="18" t="inlineStr">
         <is>
           <t>Открыть →</t>
         </is>
@@ -977,22 +1039,22 @@
       <c r="F15" s="6" t="inlineStr"/>
     </row>
     <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>T-815E59FB</t>
         </is>
       </c>
-      <c r="B16" s="17" t="inlineStr">
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>Анализ журналов и популярных событий Windows</t>
         </is>
       </c>
-      <c r="C16" s="17" t="inlineStr">
+      <c r="C16" s="19" t="inlineStr">
         <is>
           <t>ПТИБ (advance)</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="D16" s="20" t="inlineStr">
         <is>
           <t>Открыть →</t>
         </is>
@@ -1001,22 +1063,22 @@
       <c r="F16" s="6" t="inlineStr"/>
     </row>
     <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>T-E7421B02</t>
         </is>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Домены Active Directory. Доменная групповая политика</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>ПТИБ (advance)</t>
         </is>
       </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="D17" s="18" t="inlineStr">
         <is>
           <t>Открыть →</t>
         </is>
@@ -1025,22 +1087,22 @@
       <c r="F17" s="6" t="inlineStr"/>
     </row>
     <row r="18" ht="60" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>T-34BD901C</t>
         </is>
       </c>
-      <c r="B18" s="17" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>Доменная аутентификация. Типовые атаки на протоколы аутентификации</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="C18" s="19" t="inlineStr">
         <is>
           <t>ПТИБ (advance)</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="D18" s="20" t="inlineStr">
         <is>
           <t>Открыть →</t>
         </is>
@@ -1049,22 +1111,22 @@
       <c r="F18" s="6" t="inlineStr"/>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>T-2565E443</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Введение в LDAP</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>ПТИБ (advance)</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D19" s="18" t="inlineStr">
         <is>
           <t>Открыть →</t>
         </is>
@@ -1073,22 +1135,22 @@
       <c r="F19" s="6" t="inlineStr"/>
     </row>
     <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>T-2222062A</t>
         </is>
       </c>
-      <c r="B20" s="17" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Управление пользователями</t>
         </is>
       </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="C20" s="19" t="inlineStr">
         <is>
           <t>ПТИБ (advance)</t>
         </is>
       </c>
-      <c r="D20" s="18" t="inlineStr">
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>Открыть →</t>
         </is>
@@ -1097,22 +1159,22 @@
       <c r="F20" s="6" t="inlineStr"/>
     </row>
     <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>T-DF262806</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>Расследование и реагирование на атаку в инфраструктуре</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>ПТИБ (advance)</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr">
+      <c r="D21" s="18" t="inlineStr">
         <is>
           <t>Открыть →</t>
         </is>
@@ -1121,22 +1183,22 @@
       <c r="F21" s="6" t="inlineStr"/>
     </row>
     <row r="22" ht="67" customHeight="1">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>T-1EBBC04E</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B22" s="19" t="inlineStr">
         <is>
           <t>Отработка сценария «атака вируса-шифровальщика» на киберполигоне. Анализ результатов, обсуждение и разбор сценария</t>
         </is>
       </c>
-      <c r="C22" s="17" t="inlineStr">
+      <c r="C22" s="19" t="inlineStr">
         <is>
           <t>ПТИБ (advance)</t>
         </is>
       </c>
-      <c r="D22" s="18" t="inlineStr">
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>Открыть →</t>
         </is>
@@ -1161,19 +1223,19 @@
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A1:E1"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A7:F7"/>
   </mergeCells>
   <conditionalFormatting sqref="E11:E22">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="4">
       <formula>E11="Да"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11:F22">
-    <cfRule type="expression" priority="2" dxfId="1">
+    <cfRule type="expression" priority="2" dxfId="5">
       <formula>AND(E11="Частично",F11="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1205,15 +1267,15 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;CПробная версия • &amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;Crozum · Пробная версия · &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1221,7 +1283,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="0017324D"/>
+    <tabColor rgb="00221F1F"/>
     <outlinePr summaryBelow="1" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1236,7 +1298,7 @@
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1">
+    <row r="1" ht="52" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>СОДЕРЖАНИЕ ТЕМ</t>
@@ -1246,7 +1308,6 @@
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -1267,17 +1328,25 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="6" customHeight="1">
+      <c r="A4" s="14" t="n"/>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="14" t="n"/>
+      <c r="D4" s="15" t="n"/>
+      <c r="E4" s="15" t="n"/>
+      <c r="F4" s="15" t="n"/>
+    </row>
     <row r="5" ht="49" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Кибербезопасность, информационная безопасность, защита информации. Опыт противодействия киберпреступности (на примере Республики Беларусь и Российской Федерации)</t>
         </is>
       </c>
-      <c r="B5" s="20" t="n"/>
-      <c r="C5" s="20" t="n"/>
-      <c r="D5" s="20" t="n"/>
-      <c r="E5" s="20" t="n"/>
-      <c r="F5" s="20" t="n"/>
+      <c r="B5" s="22" t="n"/>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="22" t="n"/>
+      <c r="F5" s="22" t="n"/>
     </row>
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -1304,16 +1373,16 @@
       <c r="F7" s="4" t="n"/>
     </row>
     <row r="8" ht="76" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>Киберпреступность. Международный опыт противодействия киберпреступности. Построение системы обеспечения кибербезопасности в Республике Беларусь и Российской Федерации.</t>
         </is>
       </c>
-      <c r="B8" s="22" t="n"/>
-      <c r="C8" s="22" t="n"/>
-      <c r="D8" s="22" t="n"/>
-      <c r="E8" s="22" t="n"/>
-      <c r="F8" s="22" t="n"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -1334,16 +1403,16 @@
       </c>
     </row>
     <row r="12" ht="49" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>Типовая корпоративная информационная система</t>
         </is>
       </c>
-      <c r="B12" s="20" t="n"/>
-      <c r="C12" s="20" t="n"/>
-      <c r="D12" s="20" t="n"/>
-      <c r="E12" s="20" t="n"/>
-      <c r="F12" s="20" t="n"/>
+      <c r="B12" s="22" t="n"/>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="22" t="n"/>
+      <c r="E12" s="22" t="n"/>
+      <c r="F12" s="22" t="n"/>
     </row>
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -1370,16 +1439,16 @@
       <c r="F14" s="4" t="n"/>
     </row>
     <row r="15" ht="76" customHeight="1">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>Типовая корпоративная информационная система (далее – ИС), которая представляет собой комплекс программных и аппаратных средств, предназначенных для автоматизации бизнес-процессов в организации. Основные компоненты системы, структура, принципы построения и внедрения.</t>
         </is>
       </c>
-      <c r="B15" s="22" t="n"/>
-      <c r="C15" s="22" t="n"/>
-      <c r="D15" s="22" t="n"/>
-      <c r="E15" s="22" t="n"/>
-      <c r="F15" s="22" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -1400,16 +1469,16 @@
       </c>
     </row>
     <row r="19" ht="49" customHeight="1">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>Продвинутые кибератаки. Матрица MITRE ATT&amp;CK. Модель Cyber Kill Chain. Индикаторы компрометации</t>
         </is>
       </c>
-      <c r="B19" s="20" t="n"/>
-      <c r="C19" s="20" t="n"/>
-      <c r="D19" s="20" t="n"/>
-      <c r="E19" s="20" t="n"/>
-      <c r="F19" s="20" t="n"/>
+      <c r="B19" s="22" t="n"/>
+      <c r="C19" s="22" t="n"/>
+      <c r="D19" s="22" t="n"/>
+      <c r="E19" s="22" t="n"/>
+      <c r="F19" s="22" t="n"/>
     </row>
     <row r="20" ht="34" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
@@ -1436,16 +1505,16 @@
       <c r="F21" s="4" t="n"/>
     </row>
     <row r="22" ht="76" customHeight="1">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t>Матрица MITRE ATT&amp;CK. Модель Cyber Kill Chain. Детектирование инцидентов. Работа с индикаторами компрометации.</t>
         </is>
       </c>
-      <c r="B22" s="22" t="n"/>
-      <c r="C22" s="22" t="n"/>
-      <c r="D22" s="22" t="n"/>
-      <c r="E22" s="22" t="n"/>
-      <c r="F22" s="22" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
@@ -1466,16 +1535,16 @@
       </c>
     </row>
     <row r="26" ht="49" customHeight="1">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="A26" s="21" t="inlineStr">
         <is>
           <t>Современный SOC</t>
         </is>
       </c>
-      <c r="B26" s="20" t="n"/>
-      <c r="C26" s="20" t="n"/>
-      <c r="D26" s="20" t="n"/>
-      <c r="E26" s="20" t="n"/>
-      <c r="F26" s="20" t="n"/>
+      <c r="B26" s="22" t="n"/>
+      <c r="C26" s="22" t="n"/>
+      <c r="D26" s="22" t="n"/>
+      <c r="E26" s="22" t="n"/>
+      <c r="F26" s="22" t="n"/>
     </row>
     <row r="27" ht="34" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
@@ -1502,16 +1571,16 @@
       <c r="F28" s="4" t="n"/>
     </row>
     <row r="29" ht="76" customHeight="1">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>Эволюция SOC, триада (люди, процессы, технологии), уровни процессов, метрики, роли сотрудников (L1–L3, инженеры, архитектор, руководитель), RACI-матрица, технологии (SIEM, EDR/XDR, SOAR, TI), AI и Agentic SOC.</t>
         </is>
       </c>
-      <c r="B29" s="22" t="n"/>
-      <c r="C29" s="22" t="n"/>
-      <c r="D29" s="22" t="n"/>
-      <c r="E29" s="22" t="n"/>
-      <c r="F29" s="22" t="n"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
@@ -1532,16 +1601,16 @@
       </c>
     </row>
     <row r="33" ht="49" customHeight="1">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="A33" s="21" t="inlineStr">
         <is>
           <t>Жизненный цикл информационной безопасности</t>
         </is>
       </c>
-      <c r="B33" s="20" t="n"/>
-      <c r="C33" s="20" t="n"/>
-      <c r="D33" s="20" t="n"/>
-      <c r="E33" s="20" t="n"/>
-      <c r="F33" s="20" t="n"/>
+      <c r="B33" s="22" t="n"/>
+      <c r="C33" s="22" t="n"/>
+      <c r="D33" s="22" t="n"/>
+      <c r="E33" s="22" t="n"/>
+      <c r="F33" s="22" t="n"/>
     </row>
     <row r="34" ht="34" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
@@ -1568,16 +1637,16 @@
       <c r="F35" s="4" t="n"/>
     </row>
     <row r="36" ht="76" customHeight="1">
-      <c r="A36" s="21" t="inlineStr">
+      <c r="A36" s="23" t="inlineStr">
         <is>
           <t>Определения, связанные с информационной безопасностью (ИБ). Этапы жизненного цикла.</t>
         </is>
       </c>
-      <c r="B36" s="22" t="n"/>
-      <c r="C36" s="22" t="n"/>
-      <c r="D36" s="22" t="n"/>
-      <c r="E36" s="22" t="n"/>
-      <c r="F36" s="22" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
     </row>
     <row r="37" ht="28" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
@@ -1598,16 +1667,16 @@
       </c>
     </row>
     <row r="40" ht="49" customHeight="1">
-      <c r="A40" s="19" t="inlineStr">
+      <c r="A40" s="21" t="inlineStr">
         <is>
           <t>Анализ журналов и популярных событий Windows</t>
         </is>
       </c>
-      <c r="B40" s="20" t="n"/>
-      <c r="C40" s="20" t="n"/>
-      <c r="D40" s="20" t="n"/>
-      <c r="E40" s="20" t="n"/>
-      <c r="F40" s="20" t="n"/>
+      <c r="B40" s="22" t="n"/>
+      <c r="C40" s="22" t="n"/>
+      <c r="D40" s="22" t="n"/>
+      <c r="E40" s="22" t="n"/>
+      <c r="F40" s="22" t="n"/>
     </row>
     <row r="41" ht="34" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
@@ -1634,16 +1703,16 @@
       <c r="F42" s="4" t="n"/>
     </row>
     <row r="43" ht="76" customHeight="1">
-      <c r="A43" s="21" t="inlineStr">
+      <c r="A43" s="23" t="inlineStr">
         <is>
           <t>Инструменты анализа журналов Windows: Event Viewer (фильтры, XML), EvtxECmd (парсинг), Timeline Explorer (просмотр CSV), Get-WinEvent и Wevtutil (консоль), Hayabusa (поиск угроз по Sigma-правилам).</t>
         </is>
       </c>
-      <c r="B43" s="22" t="n"/>
-      <c r="C43" s="22" t="n"/>
-      <c r="D43" s="22" t="n"/>
-      <c r="E43" s="22" t="n"/>
-      <c r="F43" s="22" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
     </row>
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="3" t="inlineStr">
@@ -1664,16 +1733,16 @@
       </c>
     </row>
     <row r="47" ht="49" customHeight="1">
-      <c r="A47" s="19" t="inlineStr">
+      <c r="A47" s="21" t="inlineStr">
         <is>
           <t>Домены Active Directory. Доменная групповая политика</t>
         </is>
       </c>
-      <c r="B47" s="20" t="n"/>
-      <c r="C47" s="20" t="n"/>
-      <c r="D47" s="20" t="n"/>
-      <c r="E47" s="20" t="n"/>
-      <c r="F47" s="20" t="n"/>
+      <c r="B47" s="22" t="n"/>
+      <c r="C47" s="22" t="n"/>
+      <c r="D47" s="22" t="n"/>
+      <c r="E47" s="22" t="n"/>
+      <c r="F47" s="22" t="n"/>
     </row>
     <row r="48" ht="34" customHeight="1">
       <c r="A48" s="3" t="inlineStr">
@@ -1700,17 +1769,17 @@
       <c r="F49" s="4" t="n"/>
     </row>
     <row r="50" ht="76" customHeight="1">
-      <c r="A50" s="21" t="inlineStr">
+      <c r="A50" s="23" t="inlineStr">
         <is>
           <t>Типовая корпоративная ИС. Основные компоненты ИС, структура, принципы построения и внедрения.
 Концепция доменов в Active Directory (далее – AD). Основные принципы работы доменов, структура, роли контроллера домена.</t>
         </is>
       </c>
-      <c r="B50" s="22" t="n"/>
-      <c r="C50" s="22" t="n"/>
-      <c r="D50" s="22" t="n"/>
-      <c r="E50" s="22" t="n"/>
-      <c r="F50" s="22" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
     </row>
     <row r="51" ht="28" customHeight="1">
       <c r="A51" s="3" t="inlineStr">
@@ -1731,16 +1800,16 @@
       </c>
     </row>
     <row r="54" ht="49" customHeight="1">
-      <c r="A54" s="19" t="inlineStr">
+      <c r="A54" s="21" t="inlineStr">
         <is>
           <t>Доменная аутентификация. Типовые атаки на протоколы аутентификации</t>
         </is>
       </c>
-      <c r="B54" s="20" t="n"/>
-      <c r="C54" s="20" t="n"/>
-      <c r="D54" s="20" t="n"/>
-      <c r="E54" s="20" t="n"/>
-      <c r="F54" s="20" t="n"/>
+      <c r="B54" s="22" t="n"/>
+      <c r="C54" s="22" t="n"/>
+      <c r="D54" s="22" t="n"/>
+      <c r="E54" s="22" t="n"/>
+      <c r="F54" s="22" t="n"/>
     </row>
     <row r="55" ht="34" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
@@ -1767,16 +1836,16 @@
       <c r="F56" s="4" t="n"/>
     </row>
     <row r="57" ht="76" customHeight="1">
-      <c r="A57" s="21" t="inlineStr">
+      <c r="A57" s="23" t="inlineStr">
         <is>
           <t>Процесс аутентификации пользователей и компьютеров в домене Active Directory. Методы аутентификации, протоколы, используемые для передачи учетных данных, механизмы защиты от несанкционированного доступа.</t>
         </is>
       </c>
-      <c r="B57" s="22" t="n"/>
-      <c r="C57" s="22" t="n"/>
-      <c r="D57" s="22" t="n"/>
-      <c r="E57" s="22" t="n"/>
-      <c r="F57" s="22" t="n"/>
+      <c r="B57" s="2" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
     </row>
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
@@ -1797,16 +1866,16 @@
       </c>
     </row>
     <row r="61" ht="49" customHeight="1">
-      <c r="A61" s="19" t="inlineStr">
+      <c r="A61" s="21" t="inlineStr">
         <is>
           <t>Введение в LDAP</t>
         </is>
       </c>
-      <c r="B61" s="20" t="n"/>
-      <c r="C61" s="20" t="n"/>
-      <c r="D61" s="20" t="n"/>
-      <c r="E61" s="20" t="n"/>
-      <c r="F61" s="20" t="n"/>
+      <c r="B61" s="22" t="n"/>
+      <c r="C61" s="22" t="n"/>
+      <c r="D61" s="22" t="n"/>
+      <c r="E61" s="22" t="n"/>
+      <c r="F61" s="22" t="n"/>
     </row>
     <row r="62" ht="34" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
@@ -1833,16 +1902,16 @@
       <c r="F63" s="4" t="n"/>
     </row>
     <row r="64" ht="76" customHeight="1">
-      <c r="A64" s="21" t="inlineStr">
+      <c r="A64" s="23" t="inlineStr">
         <is>
           <t>LDAP (Lightweight Directory Access Protocol): основные понятия и принципы работы LDAP.</t>
         </is>
       </c>
-      <c r="B64" s="22" t="n"/>
-      <c r="C64" s="22" t="n"/>
-      <c r="D64" s="22" t="n"/>
-      <c r="E64" s="22" t="n"/>
-      <c r="F64" s="22" t="n"/>
+      <c r="B64" s="2" t="n"/>
+      <c r="C64" s="2" t="n"/>
+      <c r="D64" s="2" t="n"/>
+      <c r="E64" s="2" t="n"/>
+      <c r="F64" s="2" t="n"/>
     </row>
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
@@ -1863,16 +1932,16 @@
       </c>
     </row>
     <row r="68" ht="49" customHeight="1">
-      <c r="A68" s="19" t="inlineStr">
+      <c r="A68" s="21" t="inlineStr">
         <is>
           <t>Управление пользователями</t>
         </is>
       </c>
-      <c r="B68" s="20" t="n"/>
-      <c r="C68" s="20" t="n"/>
-      <c r="D68" s="20" t="n"/>
-      <c r="E68" s="20" t="n"/>
-      <c r="F68" s="20" t="n"/>
+      <c r="B68" s="22" t="n"/>
+      <c r="C68" s="22" t="n"/>
+      <c r="D68" s="22" t="n"/>
+      <c r="E68" s="22" t="n"/>
+      <c r="F68" s="22" t="n"/>
     </row>
     <row r="69" ht="34" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
@@ -1899,16 +1968,16 @@
       <c r="F70" s="4" t="n"/>
     </row>
     <row r="71" ht="76" customHeight="1">
-      <c r="A71" s="21" t="inlineStr">
+      <c r="A71" s="23" t="inlineStr">
         <is>
           <t>Создание, изменение, удаление пользователей. Ключевые объектные классы пользователей. Настройка атрибутов пользователей и групп. Использование LDIF для управления. Особенности кодирования в LDIF. Безопасность пользователей.</t>
         </is>
       </c>
-      <c r="B71" s="22" t="n"/>
-      <c r="C71" s="22" t="n"/>
-      <c r="D71" s="22" t="n"/>
-      <c r="E71" s="22" t="n"/>
-      <c r="F71" s="22" t="n"/>
+      <c r="B71" s="2" t="n"/>
+      <c r="C71" s="2" t="n"/>
+      <c r="D71" s="2" t="n"/>
+      <c r="E71" s="2" t="n"/>
+      <c r="F71" s="2" t="n"/>
     </row>
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
@@ -1929,16 +1998,16 @@
       </c>
     </row>
     <row r="75" ht="49" customHeight="1">
-      <c r="A75" s="19" t="inlineStr">
+      <c r="A75" s="21" t="inlineStr">
         <is>
           <t>Расследование и реагирование на атаку в инфраструктуре</t>
         </is>
       </c>
-      <c r="B75" s="20" t="n"/>
-      <c r="C75" s="20" t="n"/>
-      <c r="D75" s="20" t="n"/>
-      <c r="E75" s="20" t="n"/>
-      <c r="F75" s="20" t="n"/>
+      <c r="B75" s="22" t="n"/>
+      <c r="C75" s="22" t="n"/>
+      <c r="D75" s="22" t="n"/>
+      <c r="E75" s="22" t="n"/>
+      <c r="F75" s="22" t="n"/>
     </row>
     <row r="76" ht="34" customHeight="1">
       <c r="A76" s="3" t="inlineStr">
@@ -1965,16 +2034,16 @@
       <c r="F77" s="4" t="n"/>
     </row>
     <row r="78" ht="76" customHeight="1">
-      <c r="A78" s="21" t="inlineStr">
+      <c r="A78" s="23" t="inlineStr">
         <is>
           <t>Сбор и анализ артефактов инцидента на узлах и в сетевой инфраструктуре. Выявление вектора компрометации и определение последовательности действий нарушителя. Локализация инцидента, сдерживание распространения атаки и восстановление работоспособности сервисов. Отработка типового сценария расследования и реагирования на атаку.</t>
         </is>
       </c>
-      <c r="B78" s="22" t="n"/>
-      <c r="C78" s="22" t="n"/>
-      <c r="D78" s="22" t="n"/>
-      <c r="E78" s="22" t="n"/>
-      <c r="F78" s="22" t="n"/>
+      <c r="B78" s="2" t="n"/>
+      <c r="C78" s="2" t="n"/>
+      <c r="D78" s="2" t="n"/>
+      <c r="E78" s="2" t="n"/>
+      <c r="F78" s="2" t="n"/>
     </row>
     <row r="79" ht="28" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
@@ -1995,16 +2064,16 @@
       </c>
     </row>
     <row r="82" ht="49" customHeight="1">
-      <c r="A82" s="19" t="inlineStr">
+      <c r="A82" s="21" t="inlineStr">
         <is>
           <t>Отработка сценария «атака вируса-шифровальщика» на киберполигоне. Анализ результатов, обсуждение и разбор сценария</t>
         </is>
       </c>
-      <c r="B82" s="20" t="n"/>
-      <c r="C82" s="20" t="n"/>
-      <c r="D82" s="20" t="n"/>
-      <c r="E82" s="20" t="n"/>
-      <c r="F82" s="20" t="n"/>
+      <c r="B82" s="22" t="n"/>
+      <c r="C82" s="22" t="n"/>
+      <c r="D82" s="22" t="n"/>
+      <c r="E82" s="22" t="n"/>
+      <c r="F82" s="22" t="n"/>
     </row>
     <row r="83" ht="34" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
@@ -2031,7 +2100,7 @@
       <c r="F84" s="4" t="n"/>
     </row>
     <row r="85" ht="120" customHeight="1">
-      <c r="A85" s="21" t="inlineStr">
+      <c r="A85" s="23" t="inlineStr">
         <is>
           <t>Расследования инцидента «атака вируса-шифровальщика» в инфраструктуре. Идентификация всех этапов атаки, определение всех индикаторов компрометации.
 Сценарий самостоятельной работы:
@@ -2039,11 +2108,11 @@
 закрепление навыков оформления отчетных материалов по результатам расследования инцидента.</t>
         </is>
       </c>
-      <c r="B85" s="22" t="n"/>
-      <c r="C85" s="22" t="n"/>
-      <c r="D85" s="22" t="n"/>
-      <c r="E85" s="22" t="n"/>
-      <c r="F85" s="22" t="n"/>
+      <c r="B85" s="2" t="n"/>
+      <c r="C85" s="2" t="n"/>
+      <c r="D85" s="2" t="n"/>
+      <c r="E85" s="2" t="n"/>
+      <c r="F85" s="2" t="n"/>
     </row>
     <row r="86" ht="28" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
@@ -2074,6 +2143,7 @@
     <mergeCell ref="A37:F37"/>
     <mergeCell ref="A75:F75"/>
     <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A1:E1"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A50:F50"/>
     <mergeCell ref="A56:F56"/>
@@ -2130,7 +2200,6 @@
     <mergeCell ref="A82:F82"/>
     <mergeCell ref="A36:F36"/>
     <mergeCell ref="A45:C45"/>
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A70:F70"/>
     <mergeCell ref="A79:F79"/>
     <mergeCell ref="A61:F61"/>
@@ -2147,7 +2216,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;CПробная версия • &amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;Crozum · Пробная версия · &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2160,13 +2229,14 @@
     <brk id="60" min="0" max="16383" man="1"/>
     <brk id="74" min="0" max="16383" man="1"/>
   </rowBreaks>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00526779"/>
+    <tabColor rgb="0060756C"/>
     <outlinePr summaryBelow="1" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2181,7 +2251,7 @@
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1">
+    <row r="1" ht="52" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>КАК ЗАПОЛНИТЬ АНКЕТУ</t>
@@ -2191,199 +2261,206 @@
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="6" customHeight="1">
+      <c r="A2" s="14" t="n"/>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="15" t="n"/>
     </row>
     <row r="3" ht="27" customHeight="1">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>01 · Сохраните копию</t>
         </is>
       </c>
-      <c r="B3" s="20" t="n"/>
-      <c r="C3" s="20" t="n"/>
-      <c r="D3" s="20" t="n"/>
-      <c r="E3" s="20" t="n"/>
-      <c r="F3" s="20" t="n"/>
+      <c r="B3" s="22" t="n"/>
+      <c r="C3" s="22" t="n"/>
+      <c r="D3" s="22" t="n"/>
+      <c r="E3" s="22" t="n"/>
+      <c r="F3" s="22" t="n"/>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>Скачайте этот файл и откройте в Excel или LibreOffice Calc. В просмотрщике чата заполнение может быть недоступно.</t>
         </is>
       </c>
-      <c r="B4" s="22" t="n"/>
-      <c r="C4" s="22" t="n"/>
-      <c r="D4" s="22" t="n"/>
-      <c r="E4" s="22" t="n"/>
-      <c r="F4" s="22" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
     </row>
     <row r="6" ht="27" customHeight="1">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>02 · Представьтесь</t>
         </is>
       </c>
-      <c r="B6" s="20" t="n"/>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="20" t="n"/>
-      <c r="F6" s="20" t="n"/>
+      <c r="B6" s="22" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="22" t="n"/>
+      <c r="F6" s="22" t="n"/>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
-        <is>
-          <t>На листе «Выбор тем» укажите ФИО полностью. При желании добавьте дату. Заполняйте только жёлтые ячейки.</t>
-        </is>
-      </c>
-      <c r="B7" s="22" t="n"/>
-      <c r="C7" s="22" t="n"/>
-      <c r="D7" s="22" t="n"/>
-      <c r="E7" s="22" t="n"/>
-      <c r="F7" s="22" t="n"/>
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>На листе «Выбор тем» укажите ФИО полностью. При желании добавьте дату. Заполняйте только светло-зелёные ячейки.</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
     </row>
     <row r="9" ht="27" customHeight="1">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>03 · Изучите темы</t>
         </is>
       </c>
-      <c r="B9" s="20" t="n"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="n"/>
-      <c r="F9" s="20" t="n"/>
+      <c r="B9" s="22" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
+      <c r="F9" s="22" t="n"/>
     </row>
     <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>Нажмите «Открыть →» напротив темы. Содержание откроется внутри этого файла. Ссылка «← Отметить тему» вернёт к ответу.</t>
         </is>
       </c>
-      <c r="B10" s="22" t="n"/>
-      <c r="C10" s="22" t="n"/>
-      <c r="D10" s="22" t="n"/>
-      <c r="E10" s="22" t="n"/>
-      <c r="F10" s="22" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
     </row>
     <row r="12" ht="27" customHeight="1">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>04 · Сделайте выбор</t>
         </is>
       </c>
-      <c r="B12" s="20" t="n"/>
-      <c r="C12" s="20" t="n"/>
-      <c r="D12" s="20" t="n"/>
-      <c r="E12" s="20" t="n"/>
-      <c r="F12" s="20" t="n"/>
+      <c r="B12" s="22" t="n"/>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="22" t="n"/>
+      <c r="E12" s="22" t="n"/>
+      <c r="F12" s="22" t="n"/>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>«Да» — готовы читать всю тему. «Частично» — готовы читать часть: поясните, какую. Пустая ячейка означает «не указано», это не отказ.</t>
         </is>
       </c>
-      <c r="B13" s="22" t="n"/>
-      <c r="C13" s="22" t="n"/>
-      <c r="D13" s="22" t="n"/>
-      <c r="E13" s="22" t="n"/>
-      <c r="F13" s="22" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
     </row>
     <row r="15" ht="27" customHeight="1">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>05 · Сохраните результат</t>
         </is>
       </c>
-      <c r="B15" s="20" t="n"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="20" t="n"/>
-      <c r="F15" s="20" t="n"/>
+      <c r="B15" s="22" t="n"/>
+      <c r="C15" s="22" t="n"/>
+      <c r="D15" s="22" t="n"/>
+      <c r="E15" s="22" t="n"/>
+      <c r="F15" s="22" t="n"/>
     </row>
     <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="25" t="inlineStr">
         <is>
           <t>Можно вернуться позже. Когда закончите, выберите «Выбор завершён». Сохраните в формате .xlsx как «Анкета_Фамилия.xlsx».</t>
         </is>
       </c>
-      <c r="B16" s="22" t="n"/>
-      <c r="C16" s="22" t="n"/>
-      <c r="D16" s="22" t="n"/>
-      <c r="E16" s="22" t="n"/>
-      <c r="F16" s="22" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
     </row>
     <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="23" t="inlineStr">
+      <c r="A18" s="24" t="inlineStr">
         <is>
           <t>06 · Отправьте лично</t>
         </is>
       </c>
-      <c r="B18" s="20" t="n"/>
-      <c r="C18" s="20" t="n"/>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="20" t="n"/>
-      <c r="F18" s="20" t="n"/>
+      <c r="B18" s="22" t="n"/>
+      <c r="C18" s="22" t="n"/>
+      <c r="D18" s="22" t="n"/>
+      <c r="E18" s="22" t="n"/>
+      <c r="F18" s="22" t="n"/>
     </row>
     <row r="19" ht="48" customHeight="1">
-      <c r="A19" s="24" t="inlineStr">
+      <c r="A19" s="25" t="inlineStr">
         <is>
           <t>Передайте заполненный файл организатору лично. В общий чат предназначен только пустой шаблон. В файле нет ответов других преподавателей.</t>
         </is>
       </c>
-      <c r="B19" s="22" t="n"/>
-      <c r="C19" s="22" t="n"/>
-      <c r="D19" s="22" t="n"/>
-      <c r="E19" s="22" t="n"/>
-      <c r="F19" s="22" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
     </row>
     <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="23" t="inlineStr">
+      <c r="A21" s="24" t="inlineStr">
         <is>
           <t>О пробной версии</t>
         </is>
       </c>
-      <c r="B21" s="20" t="n"/>
-      <c r="C21" s="20" t="n"/>
-      <c r="D21" s="20" t="n"/>
-      <c r="E21" s="20" t="n"/>
-      <c r="F21" s="20" t="n"/>
+      <c r="B21" s="22" t="n"/>
+      <c r="C21" s="22" t="n"/>
+      <c r="D21" s="22" t="n"/>
+      <c r="E21" s="22" t="n"/>
+      <c r="F21" s="22" t="n"/>
     </row>
     <row r="22" ht="48" customHeight="1">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t>12 тем из одной локальной программы-образца ПТИБ (advance). Содержание перенесено из источника без смыслового пересказа. Папки Google Drive пока недоступны.</t>
         </is>
       </c>
-      <c r="B22" s="22" t="n"/>
-      <c r="C22" s="22" t="n"/>
-      <c r="D22" s="22" t="n"/>
-      <c r="E22" s="22" t="n"/>
-      <c r="F22" s="22" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
     </row>
     <row r="24" ht="27" customHeight="1">
-      <c r="A24" s="23" t="inlineStr">
+      <c r="A24" s="24" t="inlineStr">
         <is>
           <t>Для организатора</t>
         </is>
       </c>
-      <c r="B24" s="20" t="n"/>
-      <c r="C24" s="20" t="n"/>
-      <c r="D24" s="20" t="n"/>
-      <c r="E24" s="20" t="n"/>
-      <c r="F24" s="20" t="n"/>
+      <c r="B24" s="22" t="n"/>
+      <c r="C24" s="22" t="n"/>
+      <c r="D24" s="22" t="n"/>
+      <c r="E24" s="22" t="n"/>
+      <c r="F24" s="22" t="n"/>
     </row>
     <row r="25" ht="48" customHeight="1">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>Сводный реестр — отдельный файл. Здесь нет макросов, внешних подключений и сведений из прежней таблицы «Тема-Лектор_1».</t>
         </is>
       </c>
-      <c r="B25" s="22" t="n"/>
-      <c r="C25" s="22" t="n"/>
-      <c r="D25" s="22" t="n"/>
-      <c r="E25" s="22" t="n"/>
-      <c r="F25" s="22" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
@@ -2399,9 +2476,9 @@
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A9:F9"/>
     <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A1:E1"/>
     <mergeCell ref="A22:F22"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A4:F4"/>
@@ -2419,11 +2496,12 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;CПробная версия • &amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;Crozum · Пробная версия · &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>